<commit_message>
Add Fig 3 heatmaps/surfaces, Fig 3d scatter strip, LOOCV pipeline, and supporting scripts
- Rewrote Fig 3a/3b: 3 O2 heatmaps (Dactinomycin, Nifedipine, Mexiletine) + 3 surface plots
  with per-drug data xlsx, position enforcement in PPTX, and runtime rId mapping
- Replaced Fig 3d with 3-panel Accuracy vs AUC strip (Arrhythmia/XGBoost, Heart Damage/GaussianNB,
  Concern/GaussianNB) using all 12 equations with spectral color scheme
- Added R² bar chart rounding (2 decimal places), removed heatmap black borders
- Added sorted heatmap CSVs for all 25 drugs (Cleaned_Data/Heatmaps/)
- Added All_Equations_LOOCV pipeline and scatter plot scripts
- Added Fig 2 panel images and data files (d, g-l) with production notes
- Added helper scripts: heartrate analysis, surface feature heatmaps, 2D plots, data export
- Updated figure registry, slide layout, and PPTX slide 3 rId mapping

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Output/PowerPoint_Figures/Fig_3/Fig_3c_data.xlsx
+++ b/Output/PowerPoint_Figures/Fig_3/Fig_3c_data.xlsx
@@ -461,7 +461,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Surface 8</t>
+          <t>Cumulative Exposure</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -487,7 +487,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Surface 9</t>
+          <t>Recovery Model</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -513,7 +513,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Surface 3</t>
+          <t>Gaussian-Hill Hybrid</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -539,7 +539,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Surface 2</t>
+          <t>Bivariate Gaussian</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -565,7 +565,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Surface 5</t>
+          <t>Gaussian Ridge</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -591,7 +591,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Surface 6</t>
+          <t>Adaptive Response</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -617,7 +617,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Surface 10</t>
+          <t>Modified Hill</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -643,7 +643,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Surface 12</t>
+          <t>Dual Hill Hormesis</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -669,7 +669,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Surface 7</t>
+          <t>Biphasic Response</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -695,7 +695,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Surface 11</t>
+          <t>PKPD Elimination</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -721,7 +721,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Surface 4</t>
+          <t>Hormesis Hill</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -747,7 +747,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Surface 1</t>
+          <t>Dual Exponential</t>
         </is>
       </c>
       <c r="C13" t="n">

</xml_diff>